<commit_message>
Add Development_Fields workbook + municipal-bedrock tab on Top10
Development_Fields.xlsx - 10 development fields beyond circular-economy where
the model works (build the governance, stack the capital, steward the tail).
Scored & ranked live on MARKET/STACK/TAIL/FIT/TAILWIND/ENTRY with a Stacks sheet
detailing each field's grant/credit stack, compliance/steward tail, and PL fee
route, consistent with the verified funding architecture. Ranking: housing /
water / brownfield tie at top (4.58), then healthcare-behavioral, carbon,
broadband, manufacturing, workforce, food, renewables (sunsetting drags it).

Top10_Opportunities.xlsx - added Municipal_Bedrock sheet (Sutton, Shrewsbury,
Millbury, Fitchburg, MBI BEAD, Phillipston, Gardner) scored on the same criteria.

Both: zero formula errors. Figures illustrative; statuses verified 2026-06-03.

https://claude.ai/code/session_01NNVRfcBeiW4jRftzrwemzW
</commit_message>
<xml_diff>
--- a/docs/business/Top10_Opportunities.xlsx
+++ b/docs/business/Top10_Opportunities.xlsx
@@ -12,6 +12,7 @@
     <sheet name="Top10" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Revenue" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Action" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Municipal_Bedrock" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1922,4 +1923,362 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="7" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Municipal bedrock (MA) — context, scored the same way</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>The own-source/grant-funded MA municipal layer that runs even if the competitive layer disappears. Same six criteria &amp; weights as Top10. These are the stable counterweight to the business deals.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Opportunity</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Town / source</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>REV</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>PROB</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>RECUR</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>STRAT</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>SPEED</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>RISKADJ</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>Composite</t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>Sutton TIF / VAULT Diagnostic ($475M district)</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>Sutton (Compact grant)</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="D5" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="E5" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="F5" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="G5" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="H5" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="I5" s="7">
+        <f>C5*Inputs!$C$5+D5*Inputs!$C$6+E5*Inputs!$C$7+F5*Inputs!$C$8+G5*Inputs!$C$9+H5*Inputs!$C$10</f>
+        <v/>
+      </c>
+      <c r="J5" s="11">
+        <f>RANK(I5,$I$5:$I$11,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>Shrewsbury Municipal Fiber -&gt; retainer</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>Shrewsbury (c.30B s.7)</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="D6" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="E6" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="F6" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="G6" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="H6" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="I6" s="7">
+        <f>C6*Inputs!$C$5+D6*Inputs!$C$6+E6*Inputs!$C$7+F6*Inputs!$C$8+G6*Inputs!$C$9+H6*Inputs!$C$10</f>
+        <v/>
+      </c>
+      <c r="J6" s="11">
+        <f>RANK(I6,$I$5:$I$11,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>Millbury MS4 stormwater (replicable module)</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>Millbury</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="D7" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="E7" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="F7" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="G7" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="H7" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="I7" s="7">
+        <f>C7*Inputs!$C$5+D7*Inputs!$C$6+E7*Inputs!$C$7+F7*Inputs!$C$8+G7*Inputs!$C$9+H7*Inputs!$C$10</f>
+        <v/>
+      </c>
+      <c r="J7" s="11">
+        <f>RANK(I7,$I$5:$I$11,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>Fitchburg CIP (RFP 26-092, submitted)</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>Fitchburg (competitive)</t>
+        </is>
+      </c>
+      <c r="C8" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="D8" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="E8" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="F8" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="G8" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="H8" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="I8" s="7">
+        <f>C8*Inputs!$C$5+D8*Inputs!$C$6+E8*Inputs!$C$7+F8*Inputs!$C$8+G8*Inputs!$C$9+H8*Inputs!$C$10</f>
+        <v/>
+      </c>
+      <c r="J8" s="11">
+        <f>RANK(I8,$I$5:$I$11,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>MBI BEAD broadband RFQ (2026-MBI-08)</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>MA Broadband Institute</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="D9" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="E9" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="F9" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="G9" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="H9" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="I9" s="7">
+        <f>C9*Inputs!$C$5+D9*Inputs!$C$6+E9*Inputs!$C$7+F9*Inputs!$C$8+G9*Inputs!$C$9+H9*Inputs!$C$10</f>
+        <v/>
+      </c>
+      <c r="J9" s="11">
+        <f>RANK(I9,$I$5:$I$11,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>Phillipston website + Memorial Building</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>Phillipston</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="D10" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="E10" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="F10" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="G10" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="H10" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="I10" s="7">
+        <f>C10*Inputs!$C$5+D10*Inputs!$C$6+E10*Inputs!$C$7+F10*Inputs!$C$8+G10*Inputs!$C$9+H10*Inputs!$C$10</f>
+        <v/>
+      </c>
+      <c r="J10" s="11">
+        <f>RANK(I10,$I$5:$I$11,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>Gardner home-turf engagement (target)</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>Gardner (campaign flag)</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="D11" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="E11" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="F11" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="G11" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="H11" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="I11" s="7">
+        <f>C11*Inputs!$C$5+D11*Inputs!$C$6+E11*Inputs!$C$7+F11*Inputs!$C$8+G11*Inputs!$C$9+H11*Inputs!$C$10</f>
+        <v/>
+      </c>
+      <c r="J11" s="11">
+        <f>RANK(I11,$I$5:$I$11,0)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>